<commit_message>
Remove embedded fonts and upgrade Libreoffice version of every document
</commit_message>
<xml_diff>
--- a/documents/Lifespans in the Bible.xlsx
+++ b/documents/Lifespans in the Bible.xlsx
@@ -838,10 +838,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0207398807324925"/>
-          <c:y val="0.00867388520200256"/>
-          <c:w val="0.972663465090506"/>
-          <c:h val="0.840319012690651"/>
+          <c:x val="0.0207404280022165"/>
+          <c:y val="0.00867439017290563"/>
+          <c:w val="0.972636356439824"/>
+          <c:h val="0.840251499097631"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -1225,11 +1225,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="36003860"/>
-        <c:axId val="90724175"/>
+        <c:axId val="92971190"/>
+        <c:axId val="92321057"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36003860"/>
+        <c:axId val="92971190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1262,7 +1262,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90724175"/>
+        <c:crossAx val="92321057"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1270,7 +1270,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90724175"/>
+        <c:axId val="92321057"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1321,7 +1321,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36003860"/>
+        <c:crossAx val="92971190"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="50"/>
@@ -1359,9 +1359,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -1576,9 +1578,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>666000</xdr:colOff>
+      <xdr:colOff>665640</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>29520</xdr:rowOff>
+      <xdr:rowOff>29160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1587,7 +1589,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="38160" y="23040"/>
-        <a:ext cx="13642920" cy="6183720"/>
+        <a:ext cx="13642560" cy="6183360"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2466,7 +2468,7 @@
       <c r="D33" s="10"/>
       <c r="F33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>80</v>
       </c>
@@ -2479,7 +2481,7 @@
       <c r="D34" s="10"/>
       <c r="F34" s="10"/>
     </row>
-    <row r="35" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>82</v>
       </c>
@@ -2505,7 +2507,7 @@
       <c r="D36" s="10"/>
       <c r="F36" s="10"/>
     </row>
-    <row r="37" customFormat="false" ht="27.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>86</v>
       </c>
@@ -2518,7 +2520,7 @@
       <c r="D37" s="10"/>
       <c r="F37" s="10"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="21.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>88</v>
       </c>
@@ -2531,7 +2533,7 @@
       <c r="D38" s="10"/>
       <c r="F38" s="10"/>
     </row>
-    <row r="39" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>90</v>
       </c>
@@ -2570,7 +2572,7 @@
       <c r="D41" s="10"/>
       <c r="F41" s="10"/>
     </row>
-    <row r="42" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>96</v>
       </c>
@@ -2583,7 +2585,7 @@
       <c r="D42" s="10"/>
       <c r="F42" s="10"/>
     </row>
-    <row r="43" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>98</v>
       </c>
@@ -2596,7 +2598,7 @@
       <c r="D43" s="10"/>
       <c r="F43" s="10"/>
     </row>
-    <row r="44" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>100</v>
       </c>
@@ -2622,7 +2624,7 @@
       <c r="D45" s="10"/>
       <c r="F45" s="10"/>
     </row>
-    <row r="46" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>104</v>
       </c>
@@ -2635,7 +2637,7 @@
       <c r="D46" s="10"/>
       <c r="F46" s="10"/>
     </row>
-    <row r="47" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
         <v>106</v>
       </c>

</xml_diff>